<commit_message>
Finalizando a parte de alteração de nome e busca de arquivos na pasta
</commit_message>
<xml_diff>
--- a/comparacao_impressoras/comparacao_contadores.xlsx
+++ b/comparacao_impressoras/comparacao_contadores.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>modelo</t>
+          <t>modelo_arquivo1</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -434,15 +434,20 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>modelo_arquivo2</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>cont_atual_arquivo2</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>diferenca</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -462,17 +467,18 @@
       <c r="C2" t="n">
         <v>41810</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
         <v>42567</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>757</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -488,17 +494,18 @@
       <c r="C3" t="n">
         <v>263355</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>277217</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>13862</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -514,17 +521,18 @@
       <c r="C4" t="n">
         <v>121074</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
         <v>121695</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>621</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -540,17 +548,18 @@
       <c r="C5" t="n">
         <v>187380</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
         <v>189858</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>2478</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -566,17 +575,18 @@
       <c r="C6" t="n">
         <v>218301</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
         <v>219060</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>759</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -592,17 +602,18 @@
       <c r="C7" t="n">
         <v>155001</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
         <v>158389</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>3388</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -618,17 +629,18 @@
       <c r="C8" t="n">
         <v>195257</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
         <v>195942</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>685</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -644,17 +656,18 @@
       <c r="C9" t="n">
         <v>285405</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
         <v>289449</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>4044</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -670,13 +683,18 @@
       <c r="C10" t="n">
         <v>277524</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
         <v>277524</v>
       </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -696,17 +714,18 @@
       <c r="C11" t="n">
         <v>75142</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
         <v>75516</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>374</v>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -722,17 +741,18 @@
       <c r="C12" t="n">
         <v>194223</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
         <v>200800</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>6577</v>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -748,17 +768,18 @@
       <c r="C13" t="n">
         <v>23580</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
         <v>24408</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>828</v>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -774,17 +795,18 @@
       <c r="C14" t="n">
         <v>208032</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
         <v>209062</v>
       </c>
-      <c r="E14" t="n">
+      <c r="F14" t="n">
         <v>1030</v>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -800,17 +822,18 @@
       <c r="C15" t="n">
         <v>471406</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
         <v>475022</v>
       </c>
-      <c r="E15" t="n">
+      <c r="F15" t="n">
         <v>3616</v>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -826,17 +849,18 @@
       <c r="C16" t="n">
         <v>221314</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
         <v>224356</v>
       </c>
-      <c r="E16" t="n">
+      <c r="F16" t="n">
         <v>3042</v>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -852,17 +876,18 @@
       <c r="C17" t="n">
         <v>181737</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
         <v>182800</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>1063</v>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -878,17 +903,18 @@
       <c r="C18" t="n">
         <v>337159</v>
       </c>
-      <c r="D18" t="n">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
         <v>337376</v>
       </c>
-      <c r="E18" t="n">
+      <c r="F18" t="n">
         <v>217</v>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -904,17 +930,18 @@
       <c r="C19" t="n">
         <v>212990</v>
       </c>
-      <c r="D19" t="n">
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
         <v>213046</v>
       </c>
-      <c r="E19" t="n">
+      <c r="F19" t="n">
         <v>56</v>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -930,17 +957,18 @@
       <c r="C20" t="n">
         <v>92778</v>
       </c>
-      <c r="D20" t="n">
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
         <v>93391</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>613</v>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -956,17 +984,18 @@
       <c r="C21" t="n">
         <v>432882</v>
       </c>
-      <c r="D21" t="n">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
         <v>446244</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>13362</v>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -982,17 +1011,18 @@
       <c r="C22" t="n">
         <v>432960</v>
       </c>
-      <c r="D22" t="n">
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
         <v>434054</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>1094</v>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1008,17 +1038,18 @@
       <c r="C23" t="n">
         <v>217898</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
         <v>219140</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>1242</v>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1034,17 +1065,18 @@
       <c r="C24" t="n">
         <v>418820</v>
       </c>
-      <c r="D24" t="n">
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
         <v>419640</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>820</v>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1060,17 +1092,18 @@
       <c r="C25" t="n">
         <v>950679</v>
       </c>
-      <c r="D25" t="n">
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
         <v>951442</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>763</v>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1086,17 +1119,18 @@
       <c r="C26" t="n">
         <v>540210</v>
       </c>
-      <c r="D26" t="n">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
         <v>541610</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>1400</v>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1112,17 +1146,18 @@
       <c r="C27" t="n">
         <v>210887</v>
       </c>
-      <c r="D27" t="n">
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
         <v>221559</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>10672</v>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1138,17 +1173,18 @@
       <c r="C28" t="n">
         <v>338755</v>
       </c>
-      <c r="D28" t="n">
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
         <v>348066</v>
       </c>
-      <c r="E28" t="n">
+      <c r="F28" t="n">
         <v>9311</v>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1164,17 +1200,18 @@
       <c r="C29" t="n">
         <v>276139</v>
       </c>
-      <c r="D29" t="n">
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
         <v>281707</v>
       </c>
-      <c r="E29" t="n">
+      <c r="F29" t="n">
         <v>5568</v>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1190,17 +1227,18 @@
       <c r="C30" t="n">
         <v>375540</v>
       </c>
-      <c r="D30" t="n">
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
         <v>381065</v>
       </c>
-      <c r="E30" t="n">
+      <c r="F30" t="n">
         <v>5525</v>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1210,11 +1248,16 @@
       </c>
       <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
-      <c r="D31" t="n">
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SL-M4080FX</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
         <v>320448</v>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr">
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
         <is>
           <t>Serial ausente em um dos arquivos</t>
         </is>
@@ -1234,17 +1277,18 @@
       <c r="C32" t="n">
         <v>258246</v>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SLC-4062FX</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
         <v>260918</v>
       </c>
-      <c r="E32" t="n">
+      <c r="F32" t="n">
         <v>2672</v>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1260,17 +1304,18 @@
       <c r="C33" t="n">
         <v>70003</v>
       </c>
-      <c r="D33" t="n">
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SLC-4062FX</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
         <v>72055</v>
       </c>
-      <c r="E33" t="n">
+      <c r="F33" t="n">
         <v>2052</v>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1286,17 +1331,18 @@
       <c r="C34" t="n">
         <v>352374</v>
       </c>
-      <c r="D34" t="n">
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>SLC-4062FX</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
         <v>355982</v>
       </c>
-      <c r="E34" t="n">
+      <c r="F34" t="n">
         <v>3608</v>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1312,13 +1358,18 @@
       <c r="C35" t="n">
         <v>0</v>
       </c>
-      <c r="D35" t="n">
-        <v>0</v>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>ZT230</t>
+        </is>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1338,13 +1389,18 @@
       <c r="C36" t="n">
         <v>0</v>
       </c>
-      <c r="D36" t="n">
-        <v>0</v>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ZT230</t>
+        </is>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1358,11 +1414,16 @@
       </c>
       <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>ZT230</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
         <is>
           <t>Serial ausente em um dos arquivos</t>
         </is>
@@ -1382,13 +1443,18 @@
       <c r="C38" t="n">
         <v>0</v>
       </c>
-      <c r="D38" t="n">
-        <v>0</v>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>ZD220</t>
+        </is>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1408,13 +1474,18 @@
       <c r="C39" t="n">
         <v>0</v>
       </c>
-      <c r="D39" t="n">
-        <v>0</v>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ZD220</t>
+        </is>
       </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1434,13 +1505,18 @@
       <c r="C40" t="n">
         <v>0</v>
       </c>
-      <c r="D40" t="n">
-        <v>0</v>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>ZD220</t>
+        </is>
       </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1460,13 +1536,18 @@
       <c r="C41" t="n">
         <v>0</v>
       </c>
-      <c r="D41" t="n">
-        <v>0</v>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>ZD220</t>
+        </is>
       </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1486,13 +1567,18 @@
       <c r="C42" t="n">
         <v>0</v>
       </c>
-      <c r="D42" t="n">
-        <v>0</v>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ZD220</t>
+        </is>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1512,13 +1598,18 @@
       <c r="C43" t="n">
         <v>0</v>
       </c>
-      <c r="D43" t="n">
-        <v>0</v>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>ZD220</t>
+        </is>
       </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1538,13 +1629,18 @@
       <c r="C44" t="n">
         <v>0</v>
       </c>
-      <c r="D44" t="n">
-        <v>0</v>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ZD220</t>
+        </is>
       </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1564,13 +1660,18 @@
       <c r="C45" t="n">
         <v>0</v>
       </c>
-      <c r="D45" t="n">
-        <v>0</v>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>ZD220</t>
+        </is>
       </c>
       <c r="E45" t="n">
         <v>0</v>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1590,13 +1691,18 @@
       <c r="C46" t="n">
         <v>0</v>
       </c>
-      <c r="D46" t="n">
-        <v>0</v>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ZD220</t>
+        </is>
       </c>
       <c r="E46" t="n">
         <v>0</v>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1616,13 +1722,18 @@
       <c r="C47" t="n">
         <v>0</v>
       </c>
-      <c r="D47" t="n">
-        <v>0</v>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ZD220</t>
+        </is>
       </c>
       <c r="E47" t="n">
         <v>0</v>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="inlineStr">
         <is>
           <t>Sem alteração</t>
         </is>
@@ -1642,17 +1753,18 @@
       <c r="C48" t="n">
         <v>44792</v>
       </c>
-      <c r="D48" t="n">
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>SLC-4062FX</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
         <v>44870</v>
       </c>
-      <c r="E48" t="n">
+      <c r="F48" t="n">
         <v>78</v>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
+      <c r="G48" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>